<commit_message>
Complete Ghibli redesign: Totoro icons, forest colors, nature theme, JP quotes
</commit_message>
<xml_diff>
--- a/家庭環境調査票_completed.xlsx
+++ b/家庭環境調査票_completed.xlsx
@@ -1013,7 +1013,7 @@
       </c>
       <c r="B7" s="46" t="inlineStr">
         <is>
-          <t>伊藤　さつき</t>
+          <t>伊藤　颯希</t>
         </is>
       </c>
       <c r="C7" s="47" t="n"/>
@@ -1224,28 +1224,12 @@
       </c>
     </row>
     <row r="18" ht="22.95" customHeight="1" s="44">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>本人</t>
-        </is>
-      </c>
-      <c r="B18" s="24" t="inlineStr">
-        <is>
-          <t>伊藤 さつき</t>
-        </is>
-      </c>
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="24" t="n"/>
       <c r="C18" s="51" t="n"/>
-      <c r="D18" s="24" t="inlineStr">
-        <is>
-          <t>2022/9/29</t>
-        </is>
-      </c>
+      <c r="D18" s="24" t="n"/>
       <c r="E18" s="51" t="n"/>
-      <c r="F18" s="24" t="inlineStr">
-        <is>
-          <t>ブラッセル日本人幼稚園(年少)</t>
-        </is>
-      </c>
+      <c r="F18" s="24" t="n"/>
     </row>
     <row r="19" ht="22.95" customHeight="1" s="44">
       <c r="A19" s="2" t="n"/>

</xml_diff>